<commit_message>
chore: update record templates and remove Excel temp lock files
- Update lunch/milk/health/pickup/teeth-brushing/play-corner/student-health record templates
- Remove stray Excel ~$ temp lock files from repo
</commit_message>
<xml_diff>
--- a/image source/health_screening.xlsx
+++ b/image source/health_screening.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shifuu\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shifuu\Desktop\Project\kinder-track\image source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{207D173D-96F7-413E-A4B0-02CE79BF9922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58F3F0DB-2799-4536-BF04-454666CB2395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView showHorizontalScroll="0" showVerticalScroll="0" showSheetTabs="0" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -526,36 +526,42 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -571,12 +577,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -900,7 +900,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="32"/>
@@ -941,7 +941,7 @@
       <c r="AK1" s="32"/>
     </row>
     <row r="2" spans="1:37" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="37" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="32"/>
@@ -982,7 +982,7 @@
       <c r="AK2" s="32"/>
     </row>
     <row r="3" spans="1:37" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="37" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="32"/>
@@ -1023,63 +1023,63 @@
       <c r="AK3" s="32"/>
     </row>
     <row r="4" spans="1:37" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D4" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="E4" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="34"/>
-      <c r="N4" s="34"/>
-      <c r="O4" s="34"/>
-      <c r="P4" s="34"/>
-      <c r="Q4" s="34"/>
-      <c r="R4" s="34"/>
-      <c r="S4" s="34"/>
-      <c r="T4" s="34"/>
-      <c r="U4" s="34"/>
-      <c r="V4" s="34"/>
-      <c r="W4" s="34"/>
-      <c r="X4" s="34"/>
-      <c r="Y4" s="34"/>
-      <c r="Z4" s="34"/>
-      <c r="AA4" s="34"/>
-      <c r="AB4" s="34"/>
-      <c r="AC4" s="34"/>
-      <c r="AD4" s="34"/>
-      <c r="AE4" s="34"/>
-      <c r="AF4" s="34"/>
-      <c r="AG4" s="34"/>
-      <c r="AH4" s="34"/>
-      <c r="AI4" s="34"/>
-      <c r="AJ4" s="41" t="s">
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="35"/>
+      <c r="N4" s="35"/>
+      <c r="O4" s="35"/>
+      <c r="P4" s="35"/>
+      <c r="Q4" s="35"/>
+      <c r="R4" s="35"/>
+      <c r="S4" s="35"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="35"/>
+      <c r="V4" s="35"/>
+      <c r="W4" s="35"/>
+      <c r="X4" s="35"/>
+      <c r="Y4" s="35"/>
+      <c r="Z4" s="35"/>
+      <c r="AA4" s="35"/>
+      <c r="AB4" s="35"/>
+      <c r="AC4" s="35"/>
+      <c r="AD4" s="35"/>
+      <c r="AE4" s="35"/>
+      <c r="AF4" s="35"/>
+      <c r="AG4" s="35"/>
+      <c r="AH4" s="35"/>
+      <c r="AI4" s="35"/>
+      <c r="AJ4" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="AK4" s="37" t="s">
+      <c r="AK4" s="39" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="34"/>
-      <c r="B5" s="34"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
+      <c r="A5" s="35"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
       <c r="E5" s="1">
         <v>1</v>
       </c>
@@ -1173,8 +1173,8 @@
       <c r="AI5" s="1">
         <v>31</v>
       </c>
-      <c r="AJ5" s="34"/>
-      <c r="AK5" s="34"/>
+      <c r="AJ5" s="35"/>
+      <c r="AK5" s="35"/>
     </row>
     <row r="6" spans="1:37" ht="19.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
@@ -2937,12 +2937,12 @@
       <c r="AK45" s="8"/>
     </row>
     <row r="46" spans="1:37" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="43" t="s">
+      <c r="A46" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="B46" s="34"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
+      <c r="B46" s="35"/>
+      <c r="C46" s="35"/>
+      <c r="D46" s="35"/>
       <c r="E46" s="1">
         <f t="shared" ref="E46:AI46" si="1">COUNTIF(E6:E45,"✓")+COUNTIF(E6:E45,"v")+COUNTIF(E6:E45,"/")</f>
         <v>0</v>
@@ -3110,7 +3110,7 @@
       <c r="AK48" s="32"/>
     </row>
     <row r="50" spans="1:30" ht="22.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A50" s="31" t="s">
+      <c r="A50" s="40" t="s">
         <v>13</v>
       </c>
       <c r="B50" s="32"/>
@@ -3118,7 +3118,7 @@
       <c r="D50" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E50" s="38" t="e">
+      <c r="E50" s="33" t="e">
         <f>ปกติ / มาเรียน</f>
         <v>#NAME?</v>
       </c>
@@ -3129,7 +3129,7 @@
       <c r="K50" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="L50" s="38" t="e">
+      <c r="L50" s="33" t="e">
         <f>ป่วย / มีอาการ</f>
         <v>#NAME?</v>
       </c>
@@ -3140,7 +3140,7 @@
       <c r="R50" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="S50" s="38" t="e">
+      <c r="S50" s="33" t="e">
         <f>ขาดเรียน</f>
         <v>#NAME?</v>
       </c>
@@ -3151,7 +3151,7 @@
       <c r="Y50" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="Z50" s="38" t="e">
+      <c r="Z50" s="33" t="e">
         <f>ไม่มาด้วยเหตุพิเศษ</f>
         <v>#NAME?</v>
       </c>
@@ -3162,6 +3162,8 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="D4:D5"/>
     <mergeCell ref="A1:AK1"/>
     <mergeCell ref="S50:W50"/>
     <mergeCell ref="A46:D46"/>
@@ -3178,8 +3180,6 @@
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="E50:I50"/>
     <mergeCell ref="C4:C5"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="D4:D5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="72" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -3199,7 +3199,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="48" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="32"/>
@@ -3225,7 +3225,7 @@
       <c r="V1" s="32"/>
     </row>
     <row r="2" spans="1:22" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="37" t="s">
         <v>19</v>
       </c>
       <c r="B2" s="32"/>
@@ -3251,78 +3251,78 @@
       <c r="V2" s="32"/>
     </row>
     <row r="3" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
-      <c r="M3" s="34"/>
-      <c r="N3" s="34"/>
-      <c r="O3" s="34"/>
-      <c r="P3" s="34"/>
-      <c r="Q3" s="34"/>
-      <c r="R3" s="34"/>
-      <c r="S3" s="34"/>
-      <c r="T3" s="34"/>
-      <c r="U3" s="50" t="s">
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
+      <c r="N3" s="35"/>
+      <c r="O3" s="35"/>
+      <c r="P3" s="35"/>
+      <c r="Q3" s="35"/>
+      <c r="R3" s="35"/>
+      <c r="S3" s="35"/>
+      <c r="T3" s="35"/>
+      <c r="U3" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="V3" s="44" t="s">
+      <c r="V3" s="45" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:22" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="34"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="33" t="s">
+      <c r="A4" s="35"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="49" t="s">
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="51" t="s">
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="45" t="s">
+      <c r="J4" s="35"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="34"/>
-      <c r="N4" s="34"/>
-      <c r="O4" s="47" t="s">
+      <c r="M4" s="35"/>
+      <c r="N4" s="35"/>
+      <c r="O4" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="P4" s="34"/>
-      <c r="Q4" s="34"/>
-      <c r="R4" s="48" t="s">
+      <c r="P4" s="35"/>
+      <c r="Q4" s="35"/>
+      <c r="R4" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="S4" s="34"/>
-      <c r="T4" s="34"/>
-      <c r="U4" s="34"/>
-      <c r="V4" s="34"/>
+      <c r="S4" s="35"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="35"/>
+      <c r="V4" s="35"/>
     </row>
     <row r="5" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="34"/>
-      <c r="B5" s="34"/>
+      <c r="A5" s="35"/>
+      <c r="B5" s="35"/>
       <c r="C5" s="16" t="s">
         <v>29</v>
       </c>
@@ -3377,8 +3377,8 @@
       <c r="T5" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="U5" s="34"/>
-      <c r="V5" s="34"/>
+      <c r="U5" s="35"/>
+      <c r="V5" s="35"/>
     </row>
     <row r="6" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
@@ -4557,11 +4557,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A47:K47"/>
-    <mergeCell ref="U3:U5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="V3:V5"/>
     <mergeCell ref="A2:V2"/>
     <mergeCell ref="C3:T3"/>
     <mergeCell ref="L4:N4"/>
@@ -4571,6 +4566,11 @@
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="F4:H4"/>
+    <mergeCell ref="A47:K47"/>
+    <mergeCell ref="U3:U5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="V3:V5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4590,7 +4590,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="48" t="s">
         <v>32</v>
       </c>
       <c r="B1" s="32"/>

</xml_diff>